<commit_message>
Commit automatique via PowerShell
</commit_message>
<xml_diff>
--- a/Excel/liste_complete.xlsx
+++ b/Excel/liste_complete.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <bookViews>
-    <workbookView activeTab="-1"/>
+    <workbookView/>
   </bookViews>
   <sheets>
-    <sheet name="Export" sheetId="1" r:id="rId3"/>
+    <sheet name="Export" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Export'!$A$1:$J$132</definedName>

</xml_diff>